<commit_message>
Ajustes de calculos de retencion porcentual, persistencia en Proveedores y sincronizacion bidireccional
</commit_message>
<xml_diff>
--- a/ADMON REX.xlsx
+++ b/ADMON REX.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="96" documentId="8_{291624A6-3F6C-4D18-A25C-ADA59E993835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FA34BE0-B0F8-49E6-8852-8C30B197FFCB}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{9697CF30-101F-4501-88BA-2F18458486EE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9697CF30-101F-4501-88BA-2F18458486EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Administracion" sheetId="1" r:id="rId1"/>
@@ -2613,17 +2613,29 @@
     <xf numFmtId="164" fontId="7" fillId="14" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2637,29 +2649,17 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3012,16 +3012,16 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="122" t="s">
+      <c r="B3" s="113" t="s">
         <v>598</v>
       </c>
-      <c r="C3" s="122"/>
-      <c r="D3" s="122"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="113"/>
     </row>
     <row r="4" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="122"/>
-      <c r="C4" s="122"/>
-      <c r="D4" s="122"/>
+      <c r="B4" s="113"/>
+      <c r="C4" s="113"/>
+      <c r="D4" s="113"/>
     </row>
     <row r="5" spans="2:8" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H5" s="2"/>
@@ -3162,10 +3162,10 @@
       <c r="O1" s="14"/>
     </row>
     <row r="2" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="116"/>
+      <c r="C2" s="120"/>
       <c r="D2" s="11" t="s">
         <v>7</v>
       </c>
@@ -3193,10 +3193,10 @@
       <c r="L2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="116" t="s">
+      <c r="M2" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="N2" s="116"/>
+      <c r="N2" s="120"/>
       <c r="O2" s="11" t="s">
         <v>16</v>
       </c>
@@ -3205,8 +3205,8 @@
       <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" s="114"/>
-      <c r="C3" s="115"/>
+      <c r="B3" s="118"/>
+      <c r="C3" s="119"/>
       <c r="D3" s="14" t="s">
         <v>17</v>
       </c>
@@ -3245,8 +3245,8 @@
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="114"/>
-      <c r="C4" s="115"/>
+      <c r="B4" s="118"/>
+      <c r="C4" s="119"/>
       <c r="D4" s="14" t="s">
         <v>17</v>
       </c>
@@ -3282,8 +3282,8 @@
         <f t="shared" ref="A5:A8" si="2">A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="114"/>
-      <c r="C5" s="115"/>
+      <c r="B5" s="118"/>
+      <c r="C5" s="119"/>
       <c r="D5" s="14" t="s">
         <v>17</v>
       </c>
@@ -3319,8 +3319,8 @@
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="B6" s="114"/>
-      <c r="C6" s="115"/>
+      <c r="B6" s="118"/>
+      <c r="C6" s="119"/>
       <c r="D6" s="14" t="s">
         <v>17</v>
       </c>
@@ -3356,8 +3356,8 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="B7" s="114"/>
-      <c r="C7" s="115"/>
+      <c r="B7" s="118"/>
+      <c r="C7" s="119"/>
       <c r="D7" s="14" t="s">
         <v>17</v>
       </c>
@@ -3393,8 +3393,8 @@
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="B8" s="114"/>
-      <c r="C8" s="115"/>
+      <c r="B8" s="118"/>
+      <c r="C8" s="119"/>
       <c r="D8" s="14" t="s">
         <v>17</v>
       </c>
@@ -3430,8 +3430,8 @@
         <f>A7+1</f>
         <v>6</v>
       </c>
-      <c r="B9" s="114"/>
-      <c r="C9" s="115"/>
+      <c r="B9" s="118"/>
+      <c r="C9" s="119"/>
       <c r="D9" s="14" t="s">
         <v>17</v>
       </c>
@@ -3464,8 +3464,8 @@
         <f>A8+1</f>
         <v>7</v>
       </c>
-      <c r="B10" s="114"/>
-      <c r="C10" s="115"/>
+      <c r="B10" s="118"/>
+      <c r="C10" s="119"/>
       <c r="D10" s="14" t="s">
         <v>17</v>
       </c>
@@ -3497,8 +3497,8 @@
       <c r="A11" s="10">
         <v>8</v>
       </c>
-      <c r="B11" s="114"/>
-      <c r="C11" s="115"/>
+      <c r="B11" s="118"/>
+      <c r="C11" s="119"/>
       <c r="D11" s="14" t="s">
         <v>17</v>
       </c>
@@ -3530,8 +3530,8 @@
       <c r="A12" s="10">
         <v>9</v>
       </c>
-      <c r="B12" s="114"/>
-      <c r="C12" s="115"/>
+      <c r="B12" s="118"/>
+      <c r="C12" s="119"/>
       <c r="D12" s="14" t="s">
         <v>17</v>
       </c>
@@ -3563,8 +3563,8 @@
       <c r="A13" s="10">
         <v>10</v>
       </c>
-      <c r="B13" s="114"/>
-      <c r="C13" s="115"/>
+      <c r="B13" s="118"/>
+      <c r="C13" s="119"/>
       <c r="D13" s="14" t="s">
         <v>17</v>
       </c>
@@ -3596,8 +3596,8 @@
       <c r="A14" s="10">
         <v>11</v>
       </c>
-      <c r="B14" s="114"/>
-      <c r="C14" s="115"/>
+      <c r="B14" s="118"/>
+      <c r="C14" s="119"/>
       <c r="D14" s="14" t="s">
         <v>17</v>
       </c>
@@ -3629,8 +3629,8 @@
       <c r="A15" s="10">
         <v>12</v>
       </c>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115"/>
+      <c r="B15" s="118"/>
+      <c r="C15" s="119"/>
       <c r="D15" s="14" t="s">
         <v>17</v>
       </c>
@@ -3662,8 +3662,8 @@
       <c r="A16" s="10">
         <v>13</v>
       </c>
-      <c r="B16" s="114"/>
-      <c r="C16" s="115"/>
+      <c r="B16" s="118"/>
+      <c r="C16" s="119"/>
       <c r="D16" s="14" t="s">
         <v>17</v>
       </c>
@@ -3695,8 +3695,8 @@
       <c r="A17" s="10">
         <v>14</v>
       </c>
-      <c r="B17" s="114"/>
-      <c r="C17" s="115"/>
+      <c r="B17" s="118"/>
+      <c r="C17" s="119"/>
       <c r="D17" s="14" t="s">
         <v>17</v>
       </c>
@@ -3728,8 +3728,8 @@
       <c r="A18" s="10">
         <v>15</v>
       </c>
-      <c r="B18" s="114"/>
-      <c r="C18" s="115"/>
+      <c r="B18" s="118"/>
+      <c r="C18" s="119"/>
       <c r="D18" s="14" t="s">
         <v>17</v>
       </c>
@@ -3761,8 +3761,8 @@
       <c r="A19" s="10">
         <v>16</v>
       </c>
-      <c r="B19" s="114"/>
-      <c r="C19" s="115"/>
+      <c r="B19" s="118"/>
+      <c r="C19" s="119"/>
       <c r="D19" s="14" t="s">
         <v>17</v>
       </c>
@@ -3811,13 +3811,13 @@
         <f>SUMIF(L3:L19,"P",K3:K19)</f>
         <v>0</v>
       </c>
-      <c r="M20" s="117" t="s">
+      <c r="M20" s="121" t="s">
         <v>591</v>
       </c>
-      <c r="N20" s="117"/>
-      <c r="O20" s="117"/>
-      <c r="P20" s="117"/>
-      <c r="Q20" s="117"/>
+      <c r="N20" s="121"/>
+      <c r="O20" s="121"/>
+      <c r="P20" s="121"/>
+      <c r="Q20" s="121"/>
     </row>
     <row r="21" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="J21" s="22" t="s">
@@ -3825,10 +3825,10 @@
       </c>
     </row>
     <row r="22" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="116" t="s">
+      <c r="B22" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="116"/>
+      <c r="C22" s="120"/>
       <c r="D22" s="11" t="s">
         <v>7</v>
       </c>
@@ -3856,10 +3856,10 @@
       <c r="L22" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="M22" s="116" t="s">
+      <c r="M22" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="N22" s="116"/>
+      <c r="N22" s="120"/>
       <c r="O22" s="11" t="s">
         <v>16</v>
       </c>
@@ -4601,10 +4601,10 @@
       <c r="K43" s="10"/>
     </row>
     <row r="44" spans="1:15" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="116" t="s">
+      <c r="B44" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C44" s="116"/>
+      <c r="C44" s="120"/>
       <c r="D44" s="11" t="s">
         <v>7</v>
       </c>
@@ -4632,10 +4632,10 @@
       <c r="L44" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="M44" s="116" t="s">
+      <c r="M44" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="N44" s="116"/>
+      <c r="N44" s="120"/>
       <c r="O44" s="11" t="s">
         <v>16</v>
       </c>
@@ -5334,10 +5334,10 @@
       <c r="K65" s="10"/>
     </row>
     <row r="66" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B66" s="116" t="s">
+      <c r="B66" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C66" s="116"/>
+      <c r="C66" s="120"/>
       <c r="D66" s="11" t="s">
         <v>7</v>
       </c>
@@ -5365,10 +5365,10 @@
       <c r="L66" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="M66" s="116" t="s">
+      <c r="M66" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="N66" s="116"/>
+      <c r="N66" s="120"/>
       <c r="O66" s="11" t="s">
         <v>16</v>
       </c>
@@ -5729,10 +5729,10 @@
       <c r="K78" s="10"/>
     </row>
     <row r="79" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="119" t="s">
+      <c r="B79" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="C79" s="119"/>
+      <c r="C79" s="115"/>
       <c r="D79" s="91" t="s">
         <v>7</v>
       </c>
@@ -5760,14 +5760,14 @@
       <c r="L79" s="93" t="s">
         <v>15</v>
       </c>
-      <c r="M79" s="119" t="s">
+      <c r="M79" s="115" t="s">
         <v>6</v>
       </c>
-      <c r="N79" s="119"/>
+      <c r="N79" s="115"/>
       <c r="O79" s="91" t="s">
         <v>16</v>
       </c>
-      <c r="P79" s="110" t="s">
+      <c r="P79" s="122" t="s">
         <v>587</v>
       </c>
     </row>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="N80" s="95"/>
       <c r="O80" s="98"/>
-      <c r="P80" s="111"/>
+      <c r="P80" s="123"/>
     </row>
     <row r="81" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="10">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="N81" s="95"/>
       <c r="O81" s="98"/>
-      <c r="P81" s="111"/>
+      <c r="P81" s="123"/>
     </row>
     <row r="82" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="10">
@@ -5870,7 +5870,7 @@
       </c>
       <c r="N82" s="95"/>
       <c r="O82" s="98"/>
-      <c r="P82" s="112"/>
+      <c r="P82" s="124"/>
     </row>
     <row r="83" spans="1:18" ht="21" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="10">
@@ -6157,16 +6157,16 @@
       <c r="N92" s="102"/>
       <c r="O92" s="102"/>
       <c r="P92" s="102"/>
-      <c r="Q92" s="113" t="s">
+      <c r="Q92" s="125" t="s">
         <v>590</v>
       </c>
-      <c r="R92" s="113"/>
+      <c r="R92" s="125"/>
     </row>
     <row r="93" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="120" t="s">
+      <c r="B93" s="116" t="s">
         <v>6</v>
       </c>
-      <c r="C93" s="121"/>
+      <c r="C93" s="117"/>
       <c r="D93" s="11" t="s">
         <v>7</v>
       </c>
@@ -6201,15 +6201,15 @@
       <c r="P93" s="104" t="s">
         <v>27</v>
       </c>
-      <c r="Q93" s="113"/>
-      <c r="R93" s="113"/>
+      <c r="Q93" s="125"/>
+      <c r="R93" s="125"/>
     </row>
     <row r="94" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="10">
         <v>1</v>
       </c>
-      <c r="B94" s="118"/>
-      <c r="C94" s="118"/>
+      <c r="B94" s="114"/>
+      <c r="C94" s="114"/>
       <c r="D94" s="14" t="s">
         <v>28</v>
       </c>
@@ -6251,16 +6251,16 @@
         <f>O94*1.06</f>
         <v>1060</v>
       </c>
-      <c r="Q94" s="113"/>
-      <c r="R94" s="113"/>
+      <c r="Q94" s="125"/>
+      <c r="R94" s="125"/>
     </row>
     <row r="95" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="10">
         <f>A94+1</f>
         <v>2</v>
       </c>
-      <c r="B95" s="118"/>
-      <c r="C95" s="118"/>
+      <c r="B95" s="114"/>
+      <c r="C95" s="114"/>
       <c r="D95" s="14" t="s">
         <v>30</v>
       </c>
@@ -6304,16 +6304,16 @@
         <f t="shared" ref="P95:P98" si="18">O95*1.06</f>
         <v>1060</v>
       </c>
-      <c r="Q95" s="113"/>
-      <c r="R95" s="113"/>
+      <c r="Q95" s="125"/>
+      <c r="R95" s="125"/>
     </row>
     <row r="96" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="10">
         <f t="shared" ref="A96:A101" si="19">A95+1</f>
         <v>3</v>
       </c>
-      <c r="B96" s="118"/>
-      <c r="C96" s="118"/>
+      <c r="B96" s="114"/>
+      <c r="C96" s="114"/>
       <c r="D96" s="14" t="s">
         <v>31</v>
       </c>
@@ -6354,16 +6354,16 @@
         <f>O96*1.06</f>
         <v>1060</v>
       </c>
-      <c r="Q96" s="113"/>
-      <c r="R96" s="113"/>
+      <c r="Q96" s="125"/>
+      <c r="R96" s="125"/>
     </row>
     <row r="97" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="10">
         <f t="shared" si="19"/>
         <v>4</v>
       </c>
-      <c r="B97" s="118"/>
-      <c r="C97" s="118"/>
+      <c r="B97" s="114"/>
+      <c r="C97" s="114"/>
       <c r="D97" s="14" t="s">
         <v>32</v>
       </c>
@@ -6404,16 +6404,16 @@
         <f t="shared" si="18"/>
         <v>1060</v>
       </c>
-      <c r="Q97" s="113"/>
-      <c r="R97" s="113"/>
+      <c r="Q97" s="125"/>
+      <c r="R97" s="125"/>
     </row>
     <row r="98" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="10">
         <f t="shared" si="19"/>
         <v>5</v>
       </c>
-      <c r="B98" s="118"/>
-      <c r="C98" s="118"/>
+      <c r="B98" s="114"/>
+      <c r="C98" s="114"/>
       <c r="D98" s="14"/>
       <c r="E98" s="15">
         <f t="shared" si="20"/>
@@ -6446,16 +6446,16 @@
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="Q98" s="113"/>
-      <c r="R98" s="113"/>
+      <c r="Q98" s="125"/>
+      <c r="R98" s="125"/>
     </row>
     <row r="99" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="10">
         <f t="shared" si="19"/>
         <v>6</v>
       </c>
-      <c r="B99" s="118"/>
-      <c r="C99" s="118"/>
+      <c r="B99" s="114"/>
+      <c r="C99" s="114"/>
       <c r="D99" s="14"/>
       <c r="E99" s="15">
         <f t="shared" si="20"/>
@@ -6488,16 +6488,16 @@
         <f>O99*1.06</f>
         <v>0</v>
       </c>
-      <c r="Q99" s="113"/>
-      <c r="R99" s="113"/>
+      <c r="Q99" s="125"/>
+      <c r="R99" s="125"/>
     </row>
     <row r="100" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="10">
         <f t="shared" si="19"/>
         <v>7</v>
       </c>
-      <c r="B100" s="118"/>
-      <c r="C100" s="118"/>
+      <c r="B100" s="114"/>
+      <c r="C100" s="114"/>
       <c r="D100" s="14"/>
       <c r="E100" s="15">
         <f t="shared" si="20"/>
@@ -6532,16 +6532,16 @@
         <f t="shared" ref="P100:P101" si="22">O100*1.06</f>
         <v>0</v>
       </c>
-      <c r="Q100" s="113"/>
-      <c r="R100" s="113"/>
+      <c r="Q100" s="125"/>
+      <c r="R100" s="125"/>
     </row>
     <row r="101" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="10">
         <f t="shared" si="19"/>
         <v>8</v>
       </c>
-      <c r="B101" s="118"/>
-      <c r="C101" s="118"/>
+      <c r="B101" s="114"/>
+      <c r="C101" s="114"/>
       <c r="D101" s="14"/>
       <c r="E101" s="15">
         <f t="shared" si="20"/>
@@ -6576,8 +6576,8 @@
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="Q101" s="113"/>
-      <c r="R101" s="113"/>
+      <c r="Q101" s="125"/>
+      <c r="R101" s="125"/>
     </row>
     <row r="102" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G102" s="21">
@@ -6603,8 +6603,8 @@
       <c r="N102" s="102"/>
       <c r="O102" s="109"/>
       <c r="P102" s="109"/>
-      <c r="Q102" s="113"/>
-      <c r="R102" s="113"/>
+      <c r="Q102" s="125"/>
+      <c r="R102" s="125"/>
     </row>
     <row r="103" spans="1:18" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B103" s="10" t="s">
@@ -6625,8 +6625,8 @@
         <f>SUM(P94:P101)</f>
         <v>4240</v>
       </c>
-      <c r="Q103" s="113"/>
-      <c r="R103" s="113"/>
+      <c r="Q103" s="125"/>
+      <c r="R103" s="125"/>
     </row>
     <row r="104" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="11" t="s">
@@ -6668,8 +6668,8 @@
         <f>P103-O103</f>
         <v>240</v>
       </c>
-      <c r="Q104" s="113"/>
-      <c r="R104" s="113"/>
+      <c r="Q104" s="125"/>
+      <c r="R104" s="125"/>
     </row>
     <row r="105" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="14">
@@ -6709,8 +6709,8 @@
       <c r="P105" s="107" t="s">
         <v>28</v>
       </c>
-      <c r="Q105" s="113"/>
-      <c r="R105" s="113"/>
+      <c r="Q105" s="125"/>
+      <c r="R105" s="125"/>
     </row>
     <row r="106" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="14">
@@ -6751,8 +6751,8 @@
       <c r="P106" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="Q106" s="113"/>
-      <c r="R106" s="113"/>
+      <c r="Q106" s="125"/>
+      <c r="R106" s="125"/>
     </row>
     <row r="107" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="14">
@@ -7307,29 +7307,6 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="M79:N79"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="B96:C96"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B98:C98"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="M20:Q20"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
     <mergeCell ref="P79:P82"/>
     <mergeCell ref="Q92:R106"/>
     <mergeCell ref="B12:C12"/>
@@ -7346,6 +7323,29 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B66:C66"/>
     <mergeCell ref="M66:N66"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="M20:Q20"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="M79:N79"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B98:C98"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="B100:C100"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="60" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
@@ -7381,11 +7381,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F1" s="123" t="s">
+      <c r="F1" s="110" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="123"/>
-      <c r="H1" s="123"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
     </row>
     <row r="2" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="s">
@@ -7397,10 +7397,10 @@
       <c r="C2" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="124" t="s">
+      <c r="D2" s="111" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="125"/>
+      <c r="E2" s="112"/>
       <c r="F2" s="45" t="s">
         <v>10</v>
       </c>

</xml_diff>